<commit_message>
chore: update develop pages
</commit_message>
<xml_diff>
--- a/branches/develop/CodeSystem-mii-cs-diagnose-lebensphase-supplement-snomed.xlsx
+++ b/branches/develop/CodeSystem-mii-cs-diagnose-lebensphase-supplement-snomed.xlsx
@@ -31,7 +31,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2027.0.0-dev</t>
+    <t>2027.0.0-ballot.rc1</t>
   </si>
   <si>
     <t>Name</t>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-17</t>
+    <t>2026-09-01</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>